<commit_message>
Rename workflows-other → meshy-official-updates; hide from sidebar (visible only in All tutorials)
</commit_message>
<xml_diff>
--- a/meshy-tutorials-review.xlsx
+++ b/meshy-tutorials-review.xlsx
@@ -994,7 +994,7 @@
       <c r="G8" s="2" t="inlineStr"/>
       <c r="H8" s="9" t="inlineStr">
         <is>
-          <t>workflows-other</t>
+          <t>meshy-official-updates</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
@@ -1279,7 +1279,7 @@
       </c>
       <c r="H13" s="9" t="inlineStr">
         <is>
-          <t>workflows-other</t>
+          <t>meshy-official-updates</t>
         </is>
       </c>
       <c r="I13" s="3" t="inlineStr">
@@ -1731,7 +1731,7 @@
       <c r="G21" s="2" t="inlineStr"/>
       <c r="H21" s="9" t="inlineStr">
         <is>
-          <t>workflows-other</t>
+          <t>meshy-official-updates</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr">
@@ -1955,7 +1955,7 @@
       <c r="G25" s="2" t="inlineStr"/>
       <c r="H25" s="9" t="inlineStr">
         <is>
-          <t>workflows-other</t>
+          <t>meshy-official-updates</t>
         </is>
       </c>
       <c r="I25" s="3" t="inlineStr">
@@ -2293,7 +2293,7 @@
       <c r="G31" s="2" t="inlineStr"/>
       <c r="H31" s="9" t="inlineStr">
         <is>
-          <t>workflows-other</t>
+          <t>meshy-official-updates</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr">
@@ -2407,7 +2407,7 @@
       </c>
       <c r="H33" s="9" t="inlineStr">
         <is>
-          <t>workflows-other</t>
+          <t>meshy-official-updates</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
@@ -2635,7 +2635,7 @@
       </c>
       <c r="H37" s="9" t="inlineStr">
         <is>
-          <t>workflows-other</t>
+          <t>meshy-official-updates</t>
         </is>
       </c>
       <c r="I37" s="3" t="inlineStr">
@@ -3284,7 +3284,7 @@
   </sheetData>
   <dataValidations count="2">
     <dataValidation sqref="L2:L48" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"image-to-3d,text-to-3d,texturing,rigging,animation,multi-view,workflows-blender,workflows-unity,workflows-unreal,workflows-3d-printing,workflows-zbrush,workflows-other,api"</formula1>
+      <formula1>"image-to-3d,text-to-3d,texturing,rigging,animation,multi-view,workflows-blender,workflows-unity,workflows-unreal,workflows-3d-printing,workflows-zbrush,meshy-official-updates,api"</formula1>
     </dataValidation>
     <dataValidation sqref="K2:K48" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"keep,override,skip"</formula1>
@@ -3471,12 +3471,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>workflows-other</t>
+          <t>meshy-official-updates</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Workflows · Other (Substance / MagicaVoxel / Bambu / MCP / news / podcast / challenge)</t>
+          <t>Meshy Official Updates (HIDDEN from sidebar; surfaces under All tutorials only — for product news, podcasts, challenges, Substance/MagicaVoxel/Bambu/MCP one-offs)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
@@ -3637,7 +3637,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Workflows · Other (Substance / MagicaVoxel / Bambu / MCP / news / podcast / challenge)</t>
+          <t>Meshy Official Updates (HIDDEN from sidebar; surfaces under All tutorials only — for product news, podcasts, challenges, Substance/MagicaVoxel/Bambu/MCP one-offs)</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -3665,7 +3665,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A22"/>
+  <dimension ref="A1:A33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -3798,14 +3798,87 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Podcasts / challenges / event videos -&gt; skip (these don't belong in /tutorials).</t>
+          <t xml:space="preserve">  - Podcasts / challenges / event / product-news / one-off external-tool videos</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t xml:space="preserve">      -&gt; meshy-official-updates (hidden from sidebar, but stays in All tutorials).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
           <t xml:space="preserve">  - 3D Print + Tool combinations -&gt; workflows-3d-printing wins; tag the other tool as secondary.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>About 'meshy-official-updates' (the hidden bucket):</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - Not surfaced in the sidebar — users can't filter to it directly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - These videos still appear in the default 'All tutorials' view, sorted by date,</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    so new product announcements are still discoverable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - Use this for: Meshy 5 launch, podcasts, Halloween/Christmas challenges, Bambu/Formlabs</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    partner videos, MCP introduction, one-off Substance/MagicaVoxel tie-ins.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - When in doubt between meshy-official-updates and a feature bucket: if the video has step</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    instructions that a user follows in Meshy, use the feature bucket. If it's an</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    announcement / news / talk format, use meshy-official-updates.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v2: load all 47 videos from live API; classify on title only (in sync with xlsx)
</commit_message>
<xml_diff>
--- a/meshy-tutorials-review.xlsx
+++ b/meshy-tutorials-review.xlsx
@@ -33,7 +33,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="16">
+  <fills count="15">
     <fill>
       <patternFill/>
     </fill>
@@ -62,12 +62,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001f4d1f"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="004d3a1f"/>
+        <fgColor rgb="001f3a4d"/>
       </patternFill>
     </fill>
     <fill>
@@ -82,12 +77,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001f4d3a"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001f1f4d"/>
+        <fgColor rgb="004d3a1f"/>
       </patternFill>
     </fill>
     <fill>
@@ -102,12 +92,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001f3a4d"/>
+        <fgColor rgb="001f4d3a"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="004d1f4d"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001f1f4d"/>
       </patternFill>
     </fill>
   </fills>
@@ -137,7 +132,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -158,7 +153,6 @@
     <xf numFmtId="0" fontId="1" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="14" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="15" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -884,7 +878,7 @@
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>api</t>
+          <t>image-to-3d</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
@@ -894,7 +888,7 @@
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>developer</t>
+          <t>3D Models</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr"/>
@@ -939,9 +933,9 @@
           <t>PL9fRDm1nBS4JI0S04gYIEZlalrPz9gx23;PL9fRDm1nBS4KHZ7GCLHz8jr2WW18ggo-3</t>
         </is>
       </c>
-      <c r="H7" s="8" t="inlineStr">
-        <is>
-          <t>texturing</t>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>image-to-3d</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
@@ -951,7 +945,7 @@
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>HD Texture</t>
+          <t>(fallback)</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr"/>
@@ -992,7 +986,7 @@
         <v>16931</v>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
-      <c r="H8" s="9" t="inlineStr">
+      <c r="H8" s="8" t="inlineStr">
         <is>
           <t>meshy-official-updates</t>
         </is>
@@ -1163,7 +1157,7 @@
           <t>PL9fRDm1nBS4I1v7s5PKHVi9At7gG_iuis</t>
         </is>
       </c>
-      <c r="H11" s="10" t="inlineStr">
+      <c r="H11" s="9" t="inlineStr">
         <is>
           <t>rigging</t>
         </is>
@@ -1277,7 +1271,7 @@
           <t>PL9fRDm1nBS4I1v7s5PKHVi9At7gG_iuis</t>
         </is>
       </c>
-      <c r="H13" s="9" t="inlineStr">
+      <c r="H13" s="8" t="inlineStr">
         <is>
           <t>meshy-official-updates</t>
         </is>
@@ -1448,7 +1442,7 @@
           <t>PL9fRDm1nBS4JI0S04gYIEZlalrPz9gx23</t>
         </is>
       </c>
-      <c r="H16" s="8" t="inlineStr">
+      <c r="H16" s="10" t="inlineStr">
         <is>
           <t>texturing</t>
         </is>
@@ -1562,9 +1556,9 @@
           <t>PL9fRDm1nBS4I1v7s5PKHVi9At7gG_iuis</t>
         </is>
       </c>
-      <c r="H18" s="11" t="inlineStr">
-        <is>
-          <t>animation</t>
+      <c r="H18" s="10" t="inlineStr">
+        <is>
+          <t>texturing</t>
         </is>
       </c>
       <c r="I18" s="3" t="inlineStr">
@@ -1574,7 +1568,7 @@
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>animation</t>
+          <t>Custom Style</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr"/>
@@ -1676,9 +1670,9 @@
           <t>PL9fRDm1nBS4KHZ7GCLHz8jr2WW18ggo-3</t>
         </is>
       </c>
-      <c r="H20" s="12" t="inlineStr">
-        <is>
-          <t>workflows-unreal</t>
+      <c r="H20" s="6" t="inlineStr">
+        <is>
+          <t>workflows-blender</t>
         </is>
       </c>
       <c r="I20" s="3" t="inlineStr">
@@ -1688,7 +1682,7 @@
       </c>
       <c r="J20" s="3" t="inlineStr">
         <is>
-          <t>Unreal</t>
+          <t>Blender</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr"/>
@@ -1729,7 +1723,7 @@
         <v>302</v>
       </c>
       <c r="G21" s="2" t="inlineStr"/>
-      <c r="H21" s="9" t="inlineStr">
+      <c r="H21" s="8" t="inlineStr">
         <is>
           <t>meshy-official-updates</t>
         </is>
@@ -1786,7 +1780,7 @@
           <t>PL9fRDm1nBS4I1v7s5PKHVi9At7gG_iuis</t>
         </is>
       </c>
-      <c r="H22" s="13" t="inlineStr">
+      <c r="H22" s="11" t="inlineStr">
         <is>
           <t>multi-view</t>
         </is>
@@ -1843,9 +1837,9 @@
           <t>PL9fRDm1nBS4I1v7s5PKHVi9At7gG_iuis</t>
         </is>
       </c>
-      <c r="H23" s="11" t="inlineStr">
-        <is>
-          <t>animation</t>
+      <c r="H23" s="9" t="inlineStr">
+        <is>
+          <t>rigging</t>
         </is>
       </c>
       <c r="I23" s="3" t="inlineStr">
@@ -1855,7 +1849,7 @@
       </c>
       <c r="J23" s="3" t="inlineStr">
         <is>
-          <t>animation</t>
+          <t>Pose</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr"/>
@@ -1900,7 +1894,7 @@
           <t>PL9fRDm1nBS4JI0S04gYIEZlalrPz9gx23</t>
         </is>
       </c>
-      <c r="H24" s="14" t="inlineStr">
+      <c r="H24" s="12" t="inlineStr">
         <is>
           <t>workflows-zbrush</t>
         </is>
@@ -1953,7 +1947,7 @@
         <v>495</v>
       </c>
       <c r="G25" s="2" t="inlineStr"/>
-      <c r="H25" s="9" t="inlineStr">
+      <c r="H25" s="8" t="inlineStr">
         <is>
           <t>meshy-official-updates</t>
         </is>
@@ -2067,7 +2061,7 @@
           <t>PL9fRDm1nBS4I1v7s5PKHVi9At7gG_iuis</t>
         </is>
       </c>
-      <c r="H27" s="10" t="inlineStr">
+      <c r="H27" s="9" t="inlineStr">
         <is>
           <t>rigging</t>
         </is>
@@ -2124,7 +2118,7 @@
           <t>PL9fRDm1nBS4I1v7s5PKHVi9At7gG_iuis</t>
         </is>
       </c>
-      <c r="H28" s="8" t="inlineStr">
+      <c r="H28" s="10" t="inlineStr">
         <is>
           <t>texturing</t>
         </is>
@@ -2181,9 +2175,9 @@
           <t>PL9fRDm1nBS4JI0S04gYIEZlalrPz9gx23;PL9fRDm1nBS4I1v7s5PKHVi9At7gG_iuis</t>
         </is>
       </c>
-      <c r="H29" s="6" t="inlineStr">
-        <is>
-          <t>workflows-blender</t>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t>image-to-3d</t>
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr">
@@ -2193,7 +2187,7 @@
       </c>
       <c r="J29" s="3" t="inlineStr">
         <is>
-          <t>Blender</t>
+          <t>Meshy Tips</t>
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr"/>
@@ -2238,7 +2232,7 @@
           <t>PL9fRDm1nBS4I1v7s5PKHVi9At7gG_iuis</t>
         </is>
       </c>
-      <c r="H30" s="11" t="inlineStr">
+      <c r="H30" s="13" t="inlineStr">
         <is>
           <t>animation</t>
         </is>
@@ -2291,7 +2285,7 @@
         <v>1748</v>
       </c>
       <c r="G31" s="2" t="inlineStr"/>
-      <c r="H31" s="9" t="inlineStr">
+      <c r="H31" s="8" t="inlineStr">
         <is>
           <t>meshy-official-updates</t>
         </is>
@@ -2348,9 +2342,9 @@
           <t>PL9fRDm1nBS4I1v7s5PKHVi9At7gG_iuis</t>
         </is>
       </c>
-      <c r="H32" s="8" t="inlineStr">
-        <is>
-          <t>texturing</t>
+      <c r="H32" s="14" t="inlineStr">
+        <is>
+          <t>text-to-3d</t>
         </is>
       </c>
       <c r="I32" s="3" t="inlineStr">
@@ -2360,7 +2354,7 @@
       </c>
       <c r="J32" s="3" t="inlineStr">
         <is>
-          <t>Texture</t>
+          <t>Prompt</t>
         </is>
       </c>
       <c r="K32" s="2" t="inlineStr"/>
@@ -2405,7 +2399,7 @@
           <t>PL9fRDm1nBS4I1v7s5PKHVi9At7gG_iuis</t>
         </is>
       </c>
-      <c r="H33" s="9" t="inlineStr">
+      <c r="H33" s="8" t="inlineStr">
         <is>
           <t>meshy-official-updates</t>
         </is>
@@ -2462,7 +2456,7 @@
           <t>PL9fRDm1nBS4JI0S04gYIEZlalrPz9gx23</t>
         </is>
       </c>
-      <c r="H34" s="12" t="inlineStr">
+      <c r="H34" s="15" t="inlineStr">
         <is>
           <t>workflows-unreal</t>
         </is>
@@ -2519,7 +2513,7 @@
           <t>PL9fRDm1nBS4I1v7s5PKHVi9At7gG_iuis</t>
         </is>
       </c>
-      <c r="H35" s="15" t="inlineStr">
+      <c r="H35" s="7" t="inlineStr">
         <is>
           <t>image-to-3d</t>
         </is>
@@ -2576,7 +2570,7 @@
           <t>PL9fRDm1nBS4I1v7s5PKHVi9At7gG_iuis</t>
         </is>
       </c>
-      <c r="H36" s="8" t="inlineStr">
+      <c r="H36" s="10" t="inlineStr">
         <is>
           <t>texturing</t>
         </is>
@@ -2633,7 +2627,7 @@
           <t>PL9fRDm1nBS4I1v7s5PKHVi9At7gG_iuis</t>
         </is>
       </c>
-      <c r="H37" s="9" t="inlineStr">
+      <c r="H37" s="8" t="inlineStr">
         <is>
           <t>meshy-official-updates</t>
         </is>
@@ -2747,7 +2741,7 @@
           <t>PL9fRDm1nBS4I1v7s5PKHVi9At7gG_iuis</t>
         </is>
       </c>
-      <c r="H39" s="15" t="inlineStr">
+      <c r="H39" s="7" t="inlineStr">
         <is>
           <t>image-to-3d</t>
         </is>
@@ -2800,9 +2794,9 @@
         <v>4771</v>
       </c>
       <c r="G40" s="2" t="inlineStr"/>
-      <c r="H40" s="13" t="inlineStr">
-        <is>
-          <t>multi-view</t>
+      <c r="H40" s="10" t="inlineStr">
+        <is>
+          <t>texturing</t>
         </is>
       </c>
       <c r="I40" s="3" t="inlineStr">
@@ -2812,7 +2806,7 @@
       </c>
       <c r="J40" s="3" t="inlineStr">
         <is>
-          <t>Multi-view</t>
+          <t>PBR</t>
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr"/>
@@ -2857,7 +2851,7 @@
           <t>PL9fRDm1nBS4I1v7s5PKHVi9At7gG_iuis</t>
         </is>
       </c>
-      <c r="H41" s="15" t="inlineStr">
+      <c r="H41" s="7" t="inlineStr">
         <is>
           <t>image-to-3d</t>
         </is>
@@ -2914,7 +2908,7 @@
           <t>PL9fRDm1nBS4I1v7s5PKHVi9At7gG_iuis</t>
         </is>
       </c>
-      <c r="H42" s="15" t="inlineStr">
+      <c r="H42" s="7" t="inlineStr">
         <is>
           <t>image-to-3d</t>
         </is>
@@ -2926,7 +2920,7 @@
       </c>
       <c r="J42" s="3" t="inlineStr">
         <is>
-          <t>3D models</t>
+          <t>(fallback)</t>
         </is>
       </c>
       <c r="K42" s="2" t="inlineStr"/>
@@ -2971,9 +2965,9 @@
           <t>PL9fRDm1nBS4I1v7s5PKHVi9At7gG_iuis</t>
         </is>
       </c>
-      <c r="H43" s="11" t="inlineStr">
-        <is>
-          <t>animation</t>
+      <c r="H43" s="9" t="inlineStr">
+        <is>
+          <t>rigging</t>
         </is>
       </c>
       <c r="I43" s="3" t="inlineStr">
@@ -2983,7 +2977,7 @@
       </c>
       <c r="J43" s="3" t="inlineStr">
         <is>
-          <t>animation</t>
+          <t>Pose</t>
         </is>
       </c>
       <c r="K43" s="2" t="inlineStr"/>
@@ -3028,7 +3022,7 @@
           <t>PL9fRDm1nBS4I1v7s5PKHVi9At7gG_iuis</t>
         </is>
       </c>
-      <c r="H44" s="8" t="inlineStr">
+      <c r="H44" s="10" t="inlineStr">
         <is>
           <t>texturing</t>
         </is>
@@ -3085,9 +3079,9 @@
           <t>PL9fRDm1nBS4LE3GX01D291aTe4YxM0mIq</t>
         </is>
       </c>
-      <c r="H45" s="5" t="inlineStr">
-        <is>
-          <t>workflows-3d-printing</t>
+      <c r="H45" s="7" t="inlineStr">
+        <is>
+          <t>image-to-3d</t>
         </is>
       </c>
       <c r="I45" s="3" t="inlineStr">
@@ -3097,7 +3091,7 @@
       </c>
       <c r="J45" s="3" t="inlineStr">
         <is>
-          <t>3D print</t>
+          <t>Drawing</t>
         </is>
       </c>
       <c r="K45" s="2" t="inlineStr"/>
@@ -3142,7 +3136,7 @@
           <t>PL9fRDm1nBS4I1v7s5PKHVi9At7gG_iuis</t>
         </is>
       </c>
-      <c r="H46" s="13" t="inlineStr">
+      <c r="H46" s="11" t="inlineStr">
         <is>
           <t>multi-view</t>
         </is>
@@ -3199,7 +3193,7 @@
           <t>PL9fRDm1nBS4I1v7s5PKHVi9At7gG_iuis</t>
         </is>
       </c>
-      <c r="H47" s="16" t="inlineStr">
+      <c r="H47" s="14" t="inlineStr">
         <is>
           <t>text-to-3d</t>
         </is>
@@ -3256,9 +3250,9 @@
           <t>PL9fRDm1nBS4JI0S04gYIEZlalrPz9gx23</t>
         </is>
       </c>
-      <c r="H48" s="4" t="inlineStr">
-        <is>
-          <t>workflows-unity</t>
+      <c r="H48" s="14" t="inlineStr">
+        <is>
+          <t>text-to-3d</t>
         </is>
       </c>
       <c r="I48" s="3" t="inlineStr">
@@ -3268,7 +3262,7 @@
       </c>
       <c r="J48" s="3" t="inlineStr">
         <is>
-          <t>Unity</t>
+          <t>Stylized</t>
         </is>
       </c>
       <c r="K48" s="2" t="inlineStr"/>
@@ -3309,17 +3303,17 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="17" t="inlineStr">
+      <c r="A1" s="16" t="inlineStr">
         <is>
           <t>id (use this in column L)</t>
         </is>
       </c>
-      <c r="B1" s="17" t="inlineStr">
+      <c r="B1" s="16" t="inlineStr">
         <is>
           <t>Sidebar label</t>
         </is>
       </c>
-      <c r="C1" s="17" t="inlineStr">
+      <c r="C1" s="16" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -3513,12 +3507,12 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="17" t="inlineStr">
+      <c r="A1" s="16" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B1" s="17" t="inlineStr">
+      <c r="B1" s="16" t="inlineStr">
         <is>
           <t>Proposed count</t>
         </is>
@@ -3531,7 +3525,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3">
@@ -3541,7 +3535,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
@@ -3561,7 +3555,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -3571,7 +3565,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -3581,7 +3575,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
@@ -3601,7 +3595,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
@@ -3611,7 +3605,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -3621,7 +3615,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12">
@@ -3651,7 +3645,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>